<commit_message>
fix(finops): correct monthly summary workbook totals
</commit_message>
<xml_diff>
--- a/docs/site-monthly-costs-2026-04-28.xlsx
+++ b/docs/site-monthly-costs-2026-04-28.xlsx
@@ -2344,7 +2344,7 @@
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
     <col width="54" customWidth="1" min="2" max="2"/>
     <col width="54" customWidth="1" min="3" max="3"/>
   </cols>
@@ -2385,23 +2385,23 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Custos fixos recomendados/opcionais ligados</t>
+          <t>Custos fixos adicionais recomendados/opcionais ligados</t>
         </is>
       </c>
       <c r="B3" s="9">
-        <f>SUMPRODUCT((Custos!$E$2:$E$22&lt;&gt;"Variavel")*(Custos!$E$2:$E$22&lt;&gt;"Overage")*(Custos!$K$2:$K$22=1)*Custos!$J$2:$J$22)</f>
+        <f>SUMPRODUCT((Custos!$E$2:$E$22&lt;&gt;"Variavel")*(Custos!$E$2:$E$22&lt;&gt;"Overage")*((Custos!$D$2:$D$22="Recomendado")+(Custos!$D$2:$D$22="Opcional"))*(Custos!$K$2:$K$22=1)*Custos!$J$2:$J$22)</f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Inclui linhas opcionais marcadas em Premissas.</t>
+          <t>Mostra apenas o adicional acima do minimo obrigatorio.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Custos variaveis de pagamento no cenario atual</t>
+          <t>Custos variaveis do cenario atual</t>
         </is>
       </c>
       <c r="B4" s="9">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Baseado em pedidos, ticket e mix de pagamento das Premissas.</t>
+          <t>Inclui taxas de pagamento, storage variavel e IOF do cenario atual.</t>
         </is>
       </c>
     </row>

</xml_diff>